<commit_message>
Update vimeo_links Excel files with Lian Vimeo links.
Merge links from vimeo_metadata_export into vimeo_results.csv and regenerate vimeo_links.xlsx and vimeo_links_omit.xlsx.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/vimeo_links.xlsx
+++ b/vimeo_links.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F91"/>
+  <dimension ref="A1:F114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -551,7 +551,7 @@
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1154200765</t>
+          <t>https://vimeo.com/1154202805</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1154200948</t>
+          <t>https://vimeo.com/1154202922</t>
         </is>
       </c>
     </row>
@@ -647,7 +647,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1154203167</t>
+          <t>https://vimeo.com/1154203273</t>
         </is>
       </c>
     </row>
@@ -675,7 +675,7 @@
       <c r="E7" s="4" t="inlineStr"/>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1154203167</t>
+          <t>https://vimeo.com/1154203273</t>
         </is>
       </c>
     </row>
@@ -2859,7 +2859,7 @@
       </c>
       <c r="F80" s="7" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1177162061</t>
+          <t>https://vimeo.com/1192449734</t>
         </is>
       </c>
     </row>
@@ -2891,7 +2891,7 @@
       </c>
       <c r="F81" s="6" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1177162237</t>
+          <t>https://vimeo.com/1192449909</t>
         </is>
       </c>
     </row>
@@ -2923,7 +2923,7 @@
       </c>
       <c r="F82" s="7" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1177162517</t>
+          <t>https://vimeo.com/1192450070</t>
         </is>
       </c>
     </row>
@@ -2955,7 +2955,7 @@
       </c>
       <c r="F83" s="6" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1177162727</t>
+          <t>https://vimeo.com/1192450190</t>
         </is>
       </c>
     </row>
@@ -2987,7 +2987,7 @@
       </c>
       <c r="F84" s="7" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1192448619</t>
+          <t>https://vimeo.com/1192450344</t>
         </is>
       </c>
     </row>
@@ -3019,7 +3019,7 @@
       </c>
       <c r="F85" s="6" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1192448625</t>
+          <t>https://vimeo.com/1192450466</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="F86" s="7" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1192448633</t>
+          <t>https://vimeo.com/1192450581</t>
         </is>
       </c>
     </row>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="F87" s="6" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1192448640</t>
+          <t>https://vimeo.com/1192450716</t>
         </is>
       </c>
     </row>
@@ -3115,7 +3115,7 @@
       </c>
       <c r="F88" s="7" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1192448644</t>
+          <t>https://vimeo.com/1192450836</t>
         </is>
       </c>
     </row>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="F89" s="6" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1192448654</t>
+          <t>https://vimeo.com/1192450930</t>
         </is>
       </c>
     </row>
@@ -3211,9 +3211,689 @@
       </c>
       <c r="F91" s="6" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1192448660</t>
-        </is>
-      </c>
+          <t>https://vimeo.com/1192451107</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Makoto Aoki</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>感染症内科</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>サクラ精機株式会社</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>Case Conference: Lower Abdominal Pain, Diarrhea, Vomiting, and Lower Extremity Weakness</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>191369</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Makoto Aoki</t>
+        </is>
+      </c>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>感染症内科</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>サクラ精機株式会社</t>
+        </is>
+      </c>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>Principles of Infectious Disease Practice Part 1</t>
+        </is>
+      </c>
+      <c r="E93" s="4" t="inlineStr">
+        <is>
+          <t>497553</t>
+        </is>
+      </c>
+      <c r="F93" s="4" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Makoto Aoki</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>感染症内科</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>サクラ精機株式会社</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>Case Conference: Fever and Generalized Pain</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>191369</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Makoto Aoki</t>
+        </is>
+      </c>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t>感染症内科</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>サクラ精機株式会社</t>
+        </is>
+      </c>
+      <c r="D95" s="5" t="inlineStr">
+        <is>
+          <t>Principles of Infectious Disease Practice Part 2</t>
+        </is>
+      </c>
+      <c r="E95" s="4" t="inlineStr">
+        <is>
+          <t>497553</t>
+        </is>
+      </c>
+      <c r="F95" s="4" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Makoto Aoki</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>感染症内科</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>サクラ精機株式会社</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>Case Conference: Polydipsia, Polyuria, Dizziness, and Left Hand Pain</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>191369</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Makoto Aoki</t>
+        </is>
+      </c>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t>感染症内科</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>サクラ精機株式会社</t>
+        </is>
+      </c>
+      <c r="D97" s="5" t="inlineStr">
+        <is>
+          <t>Principles of Infectious Disease Practice Part 3</t>
+        </is>
+      </c>
+      <c r="E97" s="4" t="inlineStr">
+        <is>
+          <t>497553</t>
+        </is>
+      </c>
+      <c r="F97" s="4" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Kuo Chiang Lian</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>総合内科</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Medicine, University of Hawaii John A. Burns School of Medicine</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>34-year-old Male with Fluctuating Neuromuscular Symptoms</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>083498</t>
+        </is>
+      </c>
+      <c r="F98" s="7" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1200663950</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Kuo Chiang Lian</t>
+        </is>
+      </c>
+      <c r="B99" s="4" t="inlineStr">
+        <is>
+          <t>総合内科</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Medicine, University of Hawaii John A. Burns School of Medicine</t>
+        </is>
+      </c>
+      <c r="D99" s="5" t="inlineStr">
+        <is>
+          <t>POCUS: Applications in Hospital Medicine</t>
+        </is>
+      </c>
+      <c r="E99" s="4" t="inlineStr">
+        <is>
+          <t>585111</t>
+        </is>
+      </c>
+      <c r="F99" s="6" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1200664146</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Kuo Chiang Lian</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>総合内科</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Medicine, University of Hawaii John A. Burns School of Medicine</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>93-year-old Female with Neck pain</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>083498</t>
+        </is>
+      </c>
+      <c r="F100" s="7" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1200664284</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Kuo Chiang Lian</t>
+        </is>
+      </c>
+      <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>総合内科</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Medicine, University of Hawaii John A. Burns School of Medicine</t>
+        </is>
+      </c>
+      <c r="D101" s="5" t="inlineStr">
+        <is>
+          <t>Things We Do For No Kumu'ole (Reason) in Hospital Medicine</t>
+        </is>
+      </c>
+      <c r="E101" s="4" t="inlineStr">
+        <is>
+          <t>585111</t>
+        </is>
+      </c>
+      <c r="F101" s="6" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1200664448</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Kuo Chiang Lian</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>総合内科</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Medicine, University of Hawaii John A. Burns School of Medicine</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>Teaching How to Think: Addressing Diagnostic Error on the Wards</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>083498</t>
+        </is>
+      </c>
+      <c r="F102" s="7" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1200664576</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Kuo Chiang Lian</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>総合内科</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Medicine, University of Hawaii John A. Burns School of Medicine</t>
+        </is>
+      </c>
+      <c r="D103" s="5" t="inlineStr">
+        <is>
+          <t>Updates in Hospital Medicine: Practice Informing Articles from Late 2025</t>
+        </is>
+      </c>
+      <c r="E103" s="4" t="inlineStr">
+        <is>
+          <t>317408</t>
+        </is>
+      </c>
+      <c r="F103" s="4" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Kuo Chiang Lian</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>総合内科</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Medicine, University of Hawaii John A. Burns School of Medicine</t>
+        </is>
+      </c>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>41-year-old Male with Joint pain</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>083498</t>
+        </is>
+      </c>
+      <c r="F104" s="7" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1200664727</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Kuo Chiang Lian</t>
+        </is>
+      </c>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>総合内科</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Medicine, University of Hawaii John A. Burns School of Medicine</t>
+        </is>
+      </c>
+      <c r="D105" s="5" t="inlineStr">
+        <is>
+          <t>Do As Much Nothing As Possible: Minimizing Harm, Reducing Waste, and Maximizing Thriving in the Hospital</t>
+        </is>
+      </c>
+      <c r="E105" s="4" t="inlineStr">
+        <is>
+          <t>585111</t>
+        </is>
+      </c>
+      <c r="F105" s="6" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1200665260</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Kuo Chiang Lian</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>総合内科</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Medicine, University of Hawaii John A. Burns School of Medicine</t>
+        </is>
+      </c>
+      <c r="D106" s="3" t="inlineStr">
+        <is>
+          <t>A Woman with Fever, Rash, and Gait Disturbance</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>083498</t>
+        </is>
+      </c>
+      <c r="F106" s="7" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1200664888</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Kuo Chiang Lian</t>
+        </is>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>総合内科</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Medicine, University of Hawaii John A. Burns School of Medicine</t>
+        </is>
+      </c>
+      <c r="D107" s="5" t="inlineStr">
+        <is>
+          <t>Are You Happy? Physician Burnout and Wellness</t>
+        </is>
+      </c>
+      <c r="E107" s="4" t="inlineStr">
+        <is>
+          <t>585111</t>
+        </is>
+      </c>
+      <c r="F107" s="6" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1200665027</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Shin Miyata</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>小児外科</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>Associate Professor Pediatric General and Thoracic Surgery, SSM Health Cardinal Glennon Children's Hospital St.Louis University School of Medicine</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>Chest Wall Deformities</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>795829</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Shin Miyata</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>小児外科</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>Associate Professor Pediatric General and Thoracic Surgery, SSM Health Cardinal Glennon Children's Hospital St.Louis University School of Medicine</t>
+        </is>
+      </c>
+      <c r="D109" s="5" t="inlineStr">
+        <is>
+          <t>Emesis in children</t>
+        </is>
+      </c>
+      <c r="E109" s="4" t="inlineStr">
+        <is>
+          <t>795829</t>
+        </is>
+      </c>
+      <c r="F109" s="4" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Shin Miyata</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>小児外科</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>Associate Professor Pediatric General and Thoracic Surgery, SSM Health Cardinal Glennon Children's Hospital St.Louis University School of Medicine</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>Life and Pediatric Surgery Training of US Pediatric Surgeons: US-Japan Comparison</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>837557</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Shin Miyata</t>
+        </is>
+      </c>
+      <c r="B111" s="4" t="inlineStr">
+        <is>
+          <t>小児外科</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="inlineStr">
+        <is>
+          <t>Associate Professor Pediatric General and Thoracic Surgery, SSM Health Cardinal Glennon Children's Hospital St.Louis University School of Medicine</t>
+        </is>
+      </c>
+      <c r="D111" s="5" t="inlineStr">
+        <is>
+          <t>Pediatric Trauma</t>
+        </is>
+      </c>
+      <c r="E111" s="4" t="inlineStr">
+        <is>
+          <t>795829</t>
+        </is>
+      </c>
+      <c r="F111" s="4" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Shin Miyata</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>小児外科</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>Associate Professor Pediatric General and Thoracic Surgery, SSM Health Cardinal Glennon Children's Hospital St.Louis University School of Medicine</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>Commonな小児外科手術のHow I Do it</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>795829</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Shin Miyata</t>
+        </is>
+      </c>
+      <c r="B113" s="4" t="inlineStr">
+        <is>
+          <t>小児外科</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>Associate Professor Pediatric General and Thoracic Surgery, SSM Health Cardinal Glennon Children's Hospital St.Louis University School of Medicine</t>
+        </is>
+      </c>
+      <c r="D113" s="5" t="inlineStr">
+        <is>
+          <t>Surgery for Anorectal Malformation and Hirschsprung's Disease</t>
+        </is>
+      </c>
+      <c r="E113" s="4" t="inlineStr">
+        <is>
+          <t>795829</t>
+        </is>
+      </c>
+      <c r="F113" s="4" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Shin Miyata</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>小児外科</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>Associate Professor Pediatric General and Thoracic Surgery, SSM Health Cardinal Glennon Children's Hospital St.Louis University School of Medicine</t>
+        </is>
+      </c>
+      <c r="D114" s="3" t="inlineStr">
+        <is>
+          <t>Life and Pediatric Surgery Training of US Pediatric Surgeons: US-Japan Comparison</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>797308</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3277,6 +3957,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F89" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F90" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F91" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F98" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F99" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F100" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F101" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F102" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F104" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F105" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F106" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F107" r:id="rId69"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Publish Miyata Vimeo uploads and refresh gallery metadata.
Add five Shin Miyata lecture links from Zoom download, update vimeo_results and regenerate Excel exports for the gallery deploy workflow.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/vimeo_links.xlsx
+++ b/vimeo_links.xlsx
@@ -3629,11 +3629,7 @@
           <t>585111</t>
         </is>
       </c>
-      <c r="F105" s="6" t="inlineStr">
-        <is>
-          <t>https://vimeo.com/1200665260</t>
-        </is>
-      </c>
+      <c r="F105" s="4" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -3725,7 +3721,11 @@
           <t>795829</t>
         </is>
       </c>
-      <c r="F108" s="2" t="inlineStr"/>
+      <c r="F108" s="7" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1204023184</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
@@ -3753,7 +3753,11 @@
           <t>795829</t>
         </is>
       </c>
-      <c r="F109" s="4" t="inlineStr"/>
+      <c r="F109" s="6" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1204023395</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -3809,7 +3813,11 @@
           <t>795829</t>
         </is>
       </c>
-      <c r="F111" s="4" t="inlineStr"/>
+      <c r="F111" s="6" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1204023561</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -3837,7 +3845,11 @@
           <t>795829</t>
         </is>
       </c>
-      <c r="F112" s="2" t="inlineStr"/>
+      <c r="F112" s="7" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1204023788</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
@@ -3865,7 +3877,11 @@
           <t>795829</t>
         </is>
       </c>
-      <c r="F113" s="4" t="inlineStr"/>
+      <c r="F113" s="6" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1204024089</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -3963,9 +3979,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F101" r:id="rId64"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F102" r:id="rId65"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F104" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F105" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F106" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F107" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F106" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F107" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F108" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F109" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F111" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F112" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F113" r:id="rId73"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Kana Miyata lecture and publish to Vimeo.
Include new consultant CSV row, Zoom download result, Vimeo upload link, and refreshed gallery metadata and Excel exports.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/vimeo_links.xlsx
+++ b/vimeo_links.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F114"/>
+  <dimension ref="A1:F115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3406,7 +3406,7 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>083498</t>
+          <t>83498</t>
         </is>
       </c>
       <c r="F98" s="7" t="inlineStr">
@@ -3470,7 +3470,7 @@
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>083498</t>
+          <t>83498</t>
         </is>
       </c>
       <c r="F100" s="7" t="inlineStr">
@@ -3534,7 +3534,7 @@
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>083498</t>
+          <t>83498</t>
         </is>
       </c>
       <c r="F102" s="7" t="inlineStr">
@@ -3594,7 +3594,7 @@
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>083498</t>
+          <t>83498</t>
         </is>
       </c>
       <c r="F104" s="7" t="inlineStr">
@@ -3629,7 +3629,11 @@
           <t>585111</t>
         </is>
       </c>
-      <c r="F105" s="4" t="inlineStr"/>
+      <c r="F105" s="6" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1204027316</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -3654,7 +3658,7 @@
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>083498</t>
+          <t>83498</t>
         </is>
       </c>
       <c r="F106" s="7" t="inlineStr">
@@ -3910,6 +3914,38 @@
         </is>
       </c>
       <c r="F114" s="2" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Kana Miyata</t>
+        </is>
+      </c>
+      <c r="B115" s="4" t="inlineStr">
+        <is>
+          <t>腎臓内科</t>
+        </is>
+      </c>
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>Associate Professor Pediatric General and Thoracic Surgery, SSM Health Cardinal Glennon Children's Hospital St.Louis University School of Medicine</t>
+        </is>
+      </c>
+      <c r="D115" s="5" t="inlineStr">
+        <is>
+          <t>The Reality of Internal Medicine Training in the United States</t>
+        </is>
+      </c>
+      <c r="E115" s="4" t="inlineStr">
+        <is>
+          <t>797308</t>
+        </is>
+      </c>
+      <c r="F115" s="6" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1204027423</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3979,13 +4015,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F101" r:id="rId64"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F102" r:id="rId65"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F104" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F106" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F107" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F108" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F109" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F111" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F112" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F113" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F105" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F106" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F107" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F108" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F109" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F111" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F112" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F113" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F115" r:id="rId75"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>